<commit_message>
Configure Supabase connection and complete cloud sync for 1,230 records
</commit_message>
<xml_diff>
--- a/vendor_3.xlsx
+++ b/vendor_3.xlsx
@@ -32,6 +32,9 @@
     <t>Remarks</t>
   </si>
   <si>
+    <t>PTW NO</t>
+  </si>
+  <si>
     <t>Gaurav kumar</t>
   </si>
   <si>
@@ -53,6 +56,9 @@
     <t>Kolkata</t>
   </si>
   <si>
+    <t xml:space="preserve">Raj kumar </t>
+  </si>
+  <si>
     <t>Shyamapada Panda</t>
   </si>
   <si>
@@ -62,9 +68,6 @@
     <t>Bhubaneswar</t>
   </si>
   <si>
-    <t>PTW NO</t>
-  </si>
-  <si>
     <t>SA/WI/SD</t>
   </si>
   <si>
@@ -72,6 +75,9 @@
   </si>
   <si>
     <t>GUWAHATI</t>
+  </si>
+  <si>
+    <t>Kush kumar gupta</t>
   </si>
   <si>
     <t>SA</t>
@@ -86,10 +92,13 @@
     <t>SA/WI</t>
   </si>
   <si>
+    <t>Debasish Karmarkar</t>
+  </si>
+  <si>
     <t>Need to check</t>
   </si>
   <si>
-    <t xml:space="preserve">Raj kumar </t>
+    <t>WI/SD/ SA</t>
   </si>
   <si>
     <t>Jai  Prakash Kumar</t>
@@ -104,28 +113,37 @@
     <t>Brahmapur</t>
   </si>
   <si>
+    <t xml:space="preserve">We have use only Rourkela &amp; Sambalpur location </t>
+  </si>
+  <si>
     <t>UTKAL  KESHARI SAHOO</t>
   </si>
   <si>
     <t>Kendujhar</t>
   </si>
   <si>
+    <t>Satyabadi sahoo</t>
+  </si>
+  <si>
     <t>N</t>
   </si>
   <si>
-    <t>Kush kumar gupta</t>
+    <t>WIP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AIJIT PEGU </t>
+  </si>
+  <si>
+    <t>Guwahati</t>
   </si>
   <si>
     <t>Arindam jit</t>
   </si>
   <si>
-    <t>Debasish Karmarkar</t>
+    <t>Bikom Rabh</t>
   </si>
   <si>
     <t>Anjan Paul</t>
-  </si>
-  <si>
-    <t>WI/SD/ SA</t>
   </si>
   <si>
     <t>BBSR</t>
@@ -140,28 +158,10 @@
     <t>Sehnawaz</t>
   </si>
   <si>
-    <t xml:space="preserve">We have use only Rourkela &amp; Sambalpur location </t>
-  </si>
-  <si>
     <t>Hazaribag</t>
   </si>
   <si>
-    <t>Satyabadi sahoo</t>
-  </si>
-  <si>
     <t>Sahil</t>
-  </si>
-  <si>
-    <t>WIP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AIJIT PEGU </t>
-  </si>
-  <si>
-    <t>Guwahati</t>
-  </si>
-  <si>
-    <t>Bikom Rabh</t>
   </si>
   <si>
     <t>Site ID</t>
@@ -3225,7 +3225,7 @@
       <c r="E30" s="40"/>
       <c r="F30" s="40"/>
       <c r="G30" s="30" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="H30" s="23">
         <f t="shared" si="1"/>
@@ -3471,7 +3471,7 @@
       <c r="E35" s="40"/>
       <c r="F35" s="40"/>
       <c r="G35" s="30" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="H35" s="23">
         <f t="shared" si="1"/>
@@ -3521,7 +3521,7 @@
       <c r="E36" s="40"/>
       <c r="F36" s="40"/>
       <c r="G36" s="30" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="H36" s="23">
         <f t="shared" si="1"/>
@@ -6257,7 +6257,7 @@
       <c r="E91" s="52"/>
       <c r="F91" s="67"/>
       <c r="G91" s="50" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="H91" s="55">
         <f t="shared" si="1"/>
@@ -6303,7 +6303,7 @@
       <c r="E92" s="52"/>
       <c r="F92" s="67"/>
       <c r="G92" s="50" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="H92" s="55">
         <f t="shared" si="1"/>
@@ -6349,7 +6349,7 @@
       <c r="E93" s="52"/>
       <c r="F93" s="67"/>
       <c r="G93" s="50" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="H93" s="55">
         <f t="shared" si="1"/>
@@ -6395,7 +6395,7 @@
       <c r="E94" s="52"/>
       <c r="F94" s="67"/>
       <c r="G94" s="50" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="H94" s="55">
         <f t="shared" si="1"/>
@@ -6441,7 +6441,7 @@
       <c r="E95" s="52"/>
       <c r="F95" s="67"/>
       <c r="G95" s="50" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="H95" s="55">
         <f t="shared" si="1"/>
@@ -6487,7 +6487,7 @@
       <c r="E96" s="52"/>
       <c r="F96" s="67"/>
       <c r="G96" s="50" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="H96" s="55">
         <f t="shared" si="1"/>
@@ -6533,7 +6533,7 @@
       <c r="E97" s="52"/>
       <c r="F97" s="67"/>
       <c r="G97" s="50" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="H97" s="55">
         <f t="shared" si="1"/>
@@ -6579,7 +6579,7 @@
       <c r="E98" s="52"/>
       <c r="F98" s="67"/>
       <c r="G98" s="50" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="H98" s="55">
         <f t="shared" si="1"/>
@@ -6625,7 +6625,7 @@
       <c r="E99" s="52"/>
       <c r="F99" s="67"/>
       <c r="G99" s="50" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="H99" s="55">
         <f t="shared" si="1"/>
@@ -6671,7 +6671,7 @@
       <c r="E100" s="52"/>
       <c r="F100" s="67"/>
       <c r="G100" s="50" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="H100" s="55">
         <f t="shared" si="1"/>
@@ -6717,7 +6717,7 @@
       <c r="E101" s="52"/>
       <c r="F101" s="67"/>
       <c r="G101" s="50" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="H101" s="55">
         <f t="shared" si="1"/>
@@ -6763,7 +6763,7 @@
       <c r="E102" s="52"/>
       <c r="F102" s="67"/>
       <c r="G102" s="50" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="H102" s="55">
         <f t="shared" si="1"/>
@@ -33727,241 +33727,241 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="C4" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -33996,153 +33996,153 @@
         <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>15</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="C5" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add vendor dropdown filter to Work Order section header and fix WO status evaluation
</commit_message>
<xml_diff>
--- a/vendor_3.xlsx
+++ b/vendor_3.xlsx
@@ -32,9 +32,6 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>PTW NO</t>
-  </si>
-  <si>
     <t>Gaurav kumar</t>
   </si>
   <si>
@@ -50,16 +47,19 @@
     <t>Added</t>
   </si>
   <si>
+    <t>PTW NO</t>
+  </si>
+  <si>
     <t>Santosh Singh</t>
   </si>
   <si>
     <t>Kolkata</t>
   </si>
   <si>
-    <t xml:space="preserve">Raj kumar </t>
+    <t>Shyamapada Panda</t>
   </si>
   <si>
-    <t>Shyamapada Panda</t>
+    <t xml:space="preserve">Raj kumar </t>
   </si>
   <si>
     <t xml:space="preserve">Manoranjan kumar </t>
@@ -77,9 +77,6 @@
     <t>GUWAHATI</t>
   </si>
   <si>
-    <t>Kush kumar gupta</t>
-  </si>
-  <si>
     <t>SA</t>
   </si>
   <si>
@@ -92,13 +89,10 @@
     <t>SA/WI</t>
   </si>
   <si>
-    <t>Debasish Karmarkar</t>
-  </si>
-  <si>
     <t>Need to check</t>
   </si>
   <si>
-    <t>WI/SD/ SA</t>
+    <t>Kush kumar gupta</t>
   </si>
   <si>
     <t>Jai  Prakash Kumar</t>
@@ -107,13 +101,16 @@
     <t>Rourkela</t>
   </si>
   <si>
+    <t>Debasish Karmarkar</t>
+  </si>
+  <si>
     <t>SubhamUpadhyaya</t>
   </si>
   <si>
     <t>Brahmapur</t>
   </si>
   <si>
-    <t xml:space="preserve">We have use only Rourkela &amp; Sambalpur location </t>
+    <t>WI/SD/ SA</t>
   </si>
   <si>
     <t>UTKAL  KESHARI SAHOO</t>
@@ -122,10 +119,13 @@
     <t>Kendujhar</t>
   </si>
   <si>
-    <t>Satyabadi sahoo</t>
+    <t>N</t>
   </si>
   <si>
-    <t>N</t>
+    <t xml:space="preserve">We have use only Rourkela &amp; Sambalpur location </t>
+  </si>
+  <si>
+    <t>Satyabadi sahoo</t>
   </si>
   <si>
     <t>WIP</t>
@@ -134,10 +134,10 @@
     <t xml:space="preserve">AIJIT PEGU </t>
   </si>
   <si>
-    <t>Guwahati</t>
+    <t>Arindam jit</t>
   </si>
   <si>
-    <t>Arindam jit</t>
+    <t>Guwahati</t>
   </si>
   <si>
     <t>Bikom Rabh</t>
@@ -161,10 +161,10 @@
     <t>Hazaribag</t>
   </si>
   <si>
-    <t>Sahil</t>
+    <t>Site ID</t>
   </si>
   <si>
-    <t>Site ID</t>
+    <t>Sahil</t>
   </si>
   <si>
     <t>Site Name</t>
@@ -1737,7 +1737,7 @@
   <sheetData>
     <row r="1" ht="12.0" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>50</v>
@@ -1811,7 +1811,7 @@
       </c>
       <c r="H2" s="15">
         <f t="shared" ref="H2:H102" si="1">TODAY()-D2</f>
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="I2" s="15">
         <f t="shared" ref="I2:I102" si="2">F2-D2</f>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="H3" s="15">
         <f t="shared" si="1"/>
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="I3" s="15">
         <f t="shared" si="2"/>
@@ -1911,7 +1911,7 @@
       </c>
       <c r="H4" s="15">
         <f t="shared" si="1"/>
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="I4" s="15">
         <f t="shared" si="2"/>
@@ -1961,7 +1961,7 @@
       </c>
       <c r="H5" s="15">
         <f t="shared" si="1"/>
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="I5" s="15">
         <f t="shared" si="2"/>
@@ -2011,7 +2011,7 @@
       </c>
       <c r="H6" s="15">
         <f t="shared" si="1"/>
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="I6" s="15">
         <f t="shared" si="2"/>
@@ -2061,7 +2061,7 @@
       </c>
       <c r="H7" s="15">
         <f t="shared" si="1"/>
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="I7" s="15">
         <f t="shared" si="2"/>
@@ -2111,7 +2111,7 @@
       </c>
       <c r="H8" s="15">
         <f t="shared" si="1"/>
-        <v>444</v>
+        <v>448</v>
       </c>
       <c r="I8" s="15">
         <f t="shared" si="2"/>
@@ -2161,7 +2161,7 @@
       </c>
       <c r="H9" s="15">
         <f t="shared" si="1"/>
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="I9" s="15">
         <f t="shared" si="2"/>
@@ -2211,7 +2211,7 @@
       </c>
       <c r="H10" s="15">
         <f t="shared" si="1"/>
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="I10" s="15">
         <f t="shared" si="2"/>
@@ -2261,7 +2261,7 @@
       </c>
       <c r="H11" s="15">
         <f t="shared" si="1"/>
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="I11" s="15">
         <f t="shared" si="2"/>
@@ -2311,7 +2311,7 @@
       </c>
       <c r="H12" s="15">
         <f t="shared" si="1"/>
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="I12" s="15">
         <f t="shared" si="2"/>
@@ -2361,7 +2361,7 @@
       </c>
       <c r="H13" s="23">
         <f t="shared" si="1"/>
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="I13" s="23">
         <f t="shared" si="2"/>
@@ -2413,7 +2413,7 @@
       </c>
       <c r="H14" s="23">
         <f t="shared" si="1"/>
-        <v>419</v>
+        <v>423</v>
       </c>
       <c r="I14" s="23">
         <f t="shared" si="2"/>
@@ -2463,7 +2463,7 @@
       </c>
       <c r="H15" s="23">
         <f t="shared" si="1"/>
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="I15" s="23">
         <f t="shared" si="2"/>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="H16" s="23">
         <f t="shared" si="1"/>
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="I16" s="23">
         <f t="shared" si="2"/>
@@ -2563,7 +2563,7 @@
       </c>
       <c r="H17" s="23">
         <f t="shared" si="1"/>
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="I17" s="23">
         <f t="shared" si="2"/>
@@ -2613,7 +2613,7 @@
       </c>
       <c r="H18" s="23">
         <f t="shared" si="1"/>
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="I18" s="23">
         <f t="shared" si="2"/>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="H19" s="23">
         <f t="shared" si="1"/>
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="I19" s="23">
         <f t="shared" si="2"/>
@@ -2713,7 +2713,7 @@
       </c>
       <c r="H20" s="23">
         <f t="shared" si="1"/>
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="I20" s="23">
         <f t="shared" si="2"/>
@@ -2763,7 +2763,7 @@
       </c>
       <c r="H21" s="23">
         <f t="shared" si="1"/>
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="I21" s="23">
         <f t="shared" si="2"/>
@@ -2815,7 +2815,7 @@
       </c>
       <c r="H22" s="23">
         <f t="shared" si="1"/>
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="I22" s="23">
         <f t="shared" si="2"/>
@@ -2867,7 +2867,7 @@
       </c>
       <c r="H23" s="23">
         <f t="shared" si="1"/>
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="I23" s="23">
         <f t="shared" si="2"/>
@@ -2919,7 +2919,7 @@
       </c>
       <c r="H24" s="23">
         <f t="shared" si="1"/>
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="I24" s="23">
         <f t="shared" si="2"/>
@@ -2971,7 +2971,7 @@
       </c>
       <c r="H25" s="23">
         <f t="shared" si="1"/>
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="I25" s="23">
         <f t="shared" si="2"/>
@@ -3023,7 +3023,7 @@
       </c>
       <c r="H26" s="23">
         <f t="shared" si="1"/>
-        <v>-65351</v>
+        <v>-65347</v>
       </c>
       <c r="I26" s="23">
         <f t="shared" si="2"/>
@@ -3075,7 +3075,7 @@
       </c>
       <c r="H27" s="23">
         <f t="shared" si="1"/>
-        <v>-65351</v>
+        <v>-65347</v>
       </c>
       <c r="I27" s="23">
         <f t="shared" si="2"/>
@@ -3127,7 +3127,7 @@
       </c>
       <c r="H28" s="23">
         <f t="shared" si="1"/>
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="I28" s="23">
         <f t="shared" si="2"/>
@@ -3179,7 +3179,7 @@
       </c>
       <c r="H29" s="23">
         <f t="shared" si="1"/>
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="I29" s="23">
         <f t="shared" si="2"/>
@@ -3229,7 +3229,7 @@
       </c>
       <c r="H30" s="23">
         <f t="shared" si="1"/>
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="I30" s="23">
         <f t="shared" si="2"/>
@@ -3281,7 +3281,7 @@
       </c>
       <c r="H31" s="23">
         <f t="shared" si="1"/>
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="I31" s="23">
         <f t="shared" si="2"/>
@@ -3329,7 +3329,7 @@
       </c>
       <c r="H32" s="23">
         <f t="shared" si="1"/>
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="I32" s="23">
         <f t="shared" si="2"/>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="H33" s="23">
         <f t="shared" si="1"/>
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="I33" s="23">
         <f t="shared" si="2"/>
@@ -3427,7 +3427,7 @@
       </c>
       <c r="H34" s="23">
         <f t="shared" si="1"/>
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="I34" s="23">
         <f t="shared" si="2"/>
@@ -3475,7 +3475,7 @@
       </c>
       <c r="H35" s="23">
         <f t="shared" si="1"/>
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="I35" s="23">
         <f t="shared" si="2"/>
@@ -3525,7 +3525,7 @@
       </c>
       <c r="H36" s="23">
         <f t="shared" si="1"/>
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="I36" s="23">
         <f t="shared" si="2"/>
@@ -3577,7 +3577,7 @@
       </c>
       <c r="H37" s="23">
         <f t="shared" si="1"/>
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="I37" s="23">
         <f t="shared" si="2"/>
@@ -3627,7 +3627,7 @@
       </c>
       <c r="H38" s="23">
         <f t="shared" si="1"/>
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="I38" s="23">
         <f t="shared" si="2"/>
@@ -3673,7 +3673,7 @@
       <c r="G39" s="50"/>
       <c r="H39" s="23">
         <f t="shared" si="1"/>
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="I39" s="23">
         <f t="shared" si="2"/>
@@ -3725,7 +3725,7 @@
       </c>
       <c r="H40" s="23">
         <f t="shared" si="1"/>
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="I40" s="23">
         <f t="shared" si="2"/>
@@ -3769,7 +3769,7 @@
       <c r="G41" s="50"/>
       <c r="H41" s="23">
         <f t="shared" si="1"/>
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="I41" s="23">
         <f t="shared" si="2"/>
@@ -3819,7 +3819,7 @@
       </c>
       <c r="H42" s="23">
         <f t="shared" si="1"/>
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="I42" s="23">
         <f t="shared" si="2"/>
@@ -3869,7 +3869,7 @@
       </c>
       <c r="H43" s="23">
         <f t="shared" si="1"/>
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="I43" s="23">
         <f t="shared" si="2"/>
@@ -3919,7 +3919,7 @@
       </c>
       <c r="H44" s="23">
         <f t="shared" si="1"/>
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="I44" s="23">
         <f t="shared" si="2"/>
@@ -3969,7 +3969,7 @@
       </c>
       <c r="H45" s="23">
         <f t="shared" si="1"/>
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="I45" s="23">
         <f t="shared" si="2"/>
@@ -4019,7 +4019,7 @@
       </c>
       <c r="H46" s="23">
         <f t="shared" si="1"/>
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="I46" s="23">
         <f t="shared" si="2"/>
@@ -4071,7 +4071,7 @@
       </c>
       <c r="H47" s="23">
         <f t="shared" si="1"/>
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="I47" s="23">
         <f t="shared" si="2"/>
@@ -4121,7 +4121,7 @@
       </c>
       <c r="H48" s="23">
         <f t="shared" si="1"/>
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="I48" s="23">
         <f t="shared" si="2"/>
@@ -4171,7 +4171,7 @@
       </c>
       <c r="H49" s="23">
         <f t="shared" si="1"/>
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="I49" s="23">
         <f t="shared" si="2"/>
@@ -4223,7 +4223,7 @@
       </c>
       <c r="H50" s="23">
         <f t="shared" si="1"/>
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="I50" s="23">
         <f t="shared" si="2"/>
@@ -4273,7 +4273,7 @@
       </c>
       <c r="H51" s="23">
         <f t="shared" si="1"/>
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="I51" s="23">
         <f t="shared" si="2"/>
@@ -4325,7 +4325,7 @@
       </c>
       <c r="H52" s="23">
         <f t="shared" si="1"/>
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="I52" s="23">
         <f t="shared" si="2"/>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="H53" s="23">
         <f t="shared" si="1"/>
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="I53" s="23">
         <f t="shared" si="2"/>
@@ -4427,7 +4427,7 @@
       </c>
       <c r="H54" s="23">
         <f t="shared" si="1"/>
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="I54" s="23">
         <f t="shared" si="2"/>
@@ -4477,7 +4477,7 @@
       </c>
       <c r="H55" s="23">
         <f t="shared" si="1"/>
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="I55" s="23">
         <f t="shared" si="2"/>
@@ -4527,7 +4527,7 @@
       </c>
       <c r="H56" s="23">
         <f t="shared" si="1"/>
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="I56" s="23">
         <f t="shared" si="2"/>
@@ -4577,7 +4577,7 @@
       </c>
       <c r="H57" s="23">
         <f t="shared" si="1"/>
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="I57" s="23">
         <f t="shared" si="2"/>
@@ -4627,7 +4627,7 @@
       </c>
       <c r="H58" s="23">
         <f t="shared" si="1"/>
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="I58" s="23">
         <f t="shared" si="2"/>
@@ -4677,7 +4677,7 @@
       </c>
       <c r="H59" s="23">
         <f t="shared" si="1"/>
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="I59" s="23">
         <f t="shared" si="2"/>
@@ -4727,7 +4727,7 @@
       </c>
       <c r="H60" s="23">
         <f t="shared" si="1"/>
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="I60" s="23">
         <f t="shared" si="2"/>
@@ -4777,7 +4777,7 @@
       </c>
       <c r="H61" s="23">
         <f t="shared" si="1"/>
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="I61" s="23">
         <f t="shared" si="2"/>
@@ -4827,7 +4827,7 @@
       </c>
       <c r="H62" s="23">
         <f t="shared" si="1"/>
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="I62" s="23">
         <f t="shared" si="2"/>
@@ -4877,7 +4877,7 @@
       </c>
       <c r="H63" s="55">
         <f t="shared" si="1"/>
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="I63" s="55">
         <f t="shared" si="2"/>
@@ -4929,7 +4929,7 @@
       </c>
       <c r="H64" s="55">
         <f t="shared" si="1"/>
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="I64" s="55">
         <f t="shared" si="2"/>
@@ -4977,7 +4977,7 @@
       </c>
       <c r="H65" s="55">
         <f t="shared" si="1"/>
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="I65" s="55">
         <f t="shared" si="2"/>
@@ -5027,7 +5027,7 @@
       </c>
       <c r="H66" s="55">
         <f t="shared" si="1"/>
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="I66" s="55">
         <f t="shared" si="2"/>
@@ -5079,7 +5079,7 @@
       </c>
       <c r="H67" s="55">
         <f t="shared" si="1"/>
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="I67" s="55" t="str">
         <f t="shared" si="2"/>
@@ -5131,7 +5131,7 @@
       </c>
       <c r="H68" s="55">
         <f t="shared" si="1"/>
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="I68" s="55">
         <f t="shared" si="2"/>
@@ -5183,7 +5183,7 @@
       </c>
       <c r="H69" s="55">
         <f t="shared" si="1"/>
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="I69" s="55">
         <f t="shared" si="2"/>
@@ -5235,7 +5235,7 @@
       </c>
       <c r="H70" s="55">
         <f t="shared" si="1"/>
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="I70" s="55">
         <f t="shared" si="2"/>
@@ -5285,7 +5285,7 @@
       </c>
       <c r="H71" s="55">
         <f t="shared" si="1"/>
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="I71" s="55">
         <f t="shared" si="2"/>
@@ -5333,7 +5333,7 @@
       </c>
       <c r="H72" s="55">
         <f t="shared" si="1"/>
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="I72" s="55">
         <f t="shared" si="2"/>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="H73" s="55">
         <f t="shared" si="1"/>
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="I73" s="55">
         <f t="shared" si="2"/>
@@ -5439,7 +5439,7 @@
       </c>
       <c r="H74" s="55">
         <f t="shared" si="1"/>
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="I74" s="55">
         <f t="shared" si="2"/>
@@ -5489,7 +5489,7 @@
       </c>
       <c r="H75" s="55">
         <f t="shared" si="1"/>
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="I75" s="55">
         <f t="shared" si="2"/>
@@ -5539,7 +5539,7 @@
       </c>
       <c r="H76" s="55">
         <f t="shared" si="1"/>
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="I76" s="55">
         <f t="shared" si="2"/>
@@ -5589,7 +5589,7 @@
       </c>
       <c r="H77" s="55">
         <f t="shared" si="1"/>
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="I77" s="55">
         <f t="shared" si="2"/>
@@ -5639,7 +5639,7 @@
       </c>
       <c r="H78" s="55">
         <f t="shared" si="1"/>
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="I78" s="55">
         <f t="shared" si="2"/>
@@ -5687,7 +5687,7 @@
       </c>
       <c r="H79" s="55">
         <f t="shared" si="1"/>
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I79" s="55">
         <f t="shared" si="2"/>
@@ -5735,7 +5735,7 @@
       </c>
       <c r="H80" s="55">
         <f t="shared" si="1"/>
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I80" s="55">
         <f t="shared" si="2"/>
@@ -5783,7 +5783,7 @@
       </c>
       <c r="H81" s="55">
         <f t="shared" si="1"/>
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I81" s="55">
         <f t="shared" si="2"/>
@@ -5831,7 +5831,7 @@
       </c>
       <c r="H82" s="55">
         <f t="shared" si="1"/>
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I82" s="55">
         <f t="shared" si="2"/>
@@ -5879,7 +5879,7 @@
       </c>
       <c r="H83" s="55">
         <f t="shared" si="1"/>
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I83" s="55">
         <f t="shared" si="2"/>
@@ -5927,7 +5927,7 @@
       </c>
       <c r="H84" s="55">
         <f t="shared" si="1"/>
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I84" s="55">
         <f t="shared" si="2"/>
@@ -5975,7 +5975,7 @@
       </c>
       <c r="H85" s="55">
         <f t="shared" si="1"/>
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I85" s="55">
         <f t="shared" si="2"/>
@@ -6023,7 +6023,7 @@
       </c>
       <c r="H86" s="55">
         <f t="shared" si="1"/>
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I86" s="55">
         <f t="shared" si="2"/>
@@ -6071,7 +6071,7 @@
       </c>
       <c r="H87" s="55">
         <f t="shared" si="1"/>
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I87" s="55">
         <f t="shared" si="2"/>
@@ -6119,7 +6119,7 @@
       </c>
       <c r="H88" s="55">
         <f t="shared" si="1"/>
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I88" s="55">
         <f t="shared" si="2"/>
@@ -6167,7 +6167,7 @@
       </c>
       <c r="H89" s="55">
         <f t="shared" si="1"/>
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="I89" s="55">
         <f t="shared" si="2"/>
@@ -6215,7 +6215,7 @@
       </c>
       <c r="H90" s="55">
         <f t="shared" si="1"/>
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="I90" s="55">
         <f t="shared" si="2"/>
@@ -6261,7 +6261,7 @@
       </c>
       <c r="H91" s="55">
         <f t="shared" si="1"/>
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="I91" s="55">
         <f t="shared" si="2"/>
@@ -6307,7 +6307,7 @@
       </c>
       <c r="H92" s="55">
         <f t="shared" si="1"/>
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="I92" s="55">
         <f t="shared" si="2"/>
@@ -6353,7 +6353,7 @@
       </c>
       <c r="H93" s="55">
         <f t="shared" si="1"/>
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="I93" s="55">
         <f t="shared" si="2"/>
@@ -6399,7 +6399,7 @@
       </c>
       <c r="H94" s="55">
         <f t="shared" si="1"/>
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="I94" s="55">
         <f t="shared" si="2"/>
@@ -6445,7 +6445,7 @@
       </c>
       <c r="H95" s="55">
         <f t="shared" si="1"/>
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="I95" s="55">
         <f t="shared" si="2"/>
@@ -6491,7 +6491,7 @@
       </c>
       <c r="H96" s="55">
         <f t="shared" si="1"/>
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="I96" s="55">
         <f t="shared" si="2"/>
@@ -6537,7 +6537,7 @@
       </c>
       <c r="H97" s="55">
         <f t="shared" si="1"/>
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="I97" s="55">
         <f t="shared" si="2"/>
@@ -6583,7 +6583,7 @@
       </c>
       <c r="H98" s="55">
         <f t="shared" si="1"/>
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="I98" s="55">
         <f t="shared" si="2"/>
@@ -6629,7 +6629,7 @@
       </c>
       <c r="H99" s="55">
         <f t="shared" si="1"/>
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="I99" s="55">
         <f t="shared" si="2"/>
@@ -6675,7 +6675,7 @@
       </c>
       <c r="H100" s="55">
         <f t="shared" si="1"/>
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="I100" s="55">
         <f t="shared" si="2"/>
@@ -6721,7 +6721,7 @@
       </c>
       <c r="H101" s="55">
         <f t="shared" si="1"/>
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="I101" s="55">
         <f t="shared" si="2"/>
@@ -6767,7 +6767,7 @@
       </c>
       <c r="H102" s="55">
         <f t="shared" si="1"/>
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="I102" s="55">
         <f t="shared" si="2"/>
@@ -33727,19 +33727,19 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>9</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="3">
@@ -33750,24 +33750,24 @@
         <v>12</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -33781,7 +33781,7 @@
         <v>17</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
@@ -33792,117 +33792,117 @@
         <v>19</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="C9" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14">
@@ -33913,10 +33913,10 @@
         <v>43</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>44</v>
@@ -33930,10 +33930,10 @@
         <v>43</v>
       </c>
       <c r="C15" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="16">
@@ -33944,24 +33944,24 @@
         <v>47</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -33996,35 +33996,35 @@
         <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="4">
@@ -34035,86 +34035,86 @@
         <v>12</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>37</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10">
@@ -34122,13 +34122,13 @@
         <v>38</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="11">
@@ -34136,13 +34136,13 @@
         <v>41</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>